<commit_message>
now its all perfectly working
</commit_message>
<xml_diff>
--- a/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_BatchBA1_Attendance.xlsx
+++ b/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_BatchBA1_Attendance.xlsx
@@ -1285,7 +1285,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
@@ -1301,7 +1301,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -1317,7 +1317,7 @@
         <v>12</v>
       </c>
       <c r="D9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
@@ -1333,7 +1333,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -1509,7 +1509,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -1525,7 +1525,7 @@
         <v>12</v>
       </c>
       <c r="D22" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -1573,7 +1573,7 @@
         <v>4</v>
       </c>
       <c r="D25" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -1589,7 +1589,7 @@
         <v>12</v>
       </c>
       <c r="D26" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -5170,6 +5170,6 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>